<commit_message>
fix: improve live conversation routing and knowledge relevance
</commit_message>
<xml_diff>
--- a/artifacts/ANCFZ_Intent_Catalog_Executable_Proposal_2026-10-28.xlsx
+++ b/artifacts/ANCFZ_Intent_Catalog_Executable_Proposal_2026-10-28.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R68d6e4fb58024327"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Findings" sheetId="2" r:id="Re8c1618525fa45fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="n8n Workflow Plan" sheetId="3" r:id="R0f3c78ffd13140fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="End-to-End Flow" sheetId="4" r:id="R7c562cd0a3464a4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intent Routing Review" sheetId="5" r:id="R3687080efd2a4029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposed Requirements" sheetId="6" r:id="R642c0e6ba1eb4794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Tests" sheetId="7" r:id="R39850e98c92947f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="8" r:id="Rb82ff9de23944499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="9" r:id="Re52fcf471ae8431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="10" r:id="R66b1c8fae6724ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="11" r:id="R27d8dfc2adcf421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="12" r:id="Rc7b2a07440744228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentPolicies" sheetId="13" r:id="R9298af697d194d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentSettings" sheetId="14" r:id="R139e6ba982e549c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualityRules" sheetId="15" r:id="Rf08df1fbd7bc4fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="16" r:id="R2893ff663a864455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyRequirements" sheetId="17" r:id="Rf04be970615c4626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyTransitions" sheetId="18" r:id="R81da36d274b14b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R7a7f447ad0394a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Findings" sheetId="2" r:id="R1e4f54150bb244a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="n8n Workflow Plan" sheetId="3" r:id="R248e691f414e4506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="End-to-End Flow" sheetId="4" r:id="Rfe578583af414258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intent Routing Review" sheetId="5" r:id="R16ca87b444c647e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposed Requirements" sheetId="6" r:id="R9e6b037d8a44409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Tests" sheetId="7" r:id="R9bd46e7b85704758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="8" r:id="R4b251b35f45440c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="9" r:id="R67cb2bde3589463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="10" r:id="R23f8a66e50154c25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="11" r:id="R6ebfa7f0c82e4c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="12" r:id="Rf2053c38eb364e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentPolicies" sheetId="13" r:id="R49931d173f474c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentSettings" sheetId="14" r:id="R3e09a85902744918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualityRules" sheetId="15" r:id="Rd87bafac8aab4a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="16" r:id="Rda1fdcd2dc9c4fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyRequirements" sheetId="17" r:id="R61f62e0c57eb4212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyTransitions" sheetId="18" r:id="R7c0806a47e3c4e4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10219,6 +10219,213 @@
         <x:v>anc.clarify_primary_requirement</x:v>
       </x:c>
     </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>anc.activity.eligibility</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>anc.activity.it_software</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>anc.activity.consulting</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>anc.activity.marketing</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>anc.activity.trading</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>anc.activity.logistics</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>anc.activity.accounting</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>anc.activity.ai_blockchain</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>anc.setup.new_company</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>anc.activity.real_estate_services</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>activity</x:v>
+      </x:c>
+      <x:c r="E37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>anc.clarify_primary_requirement</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12326,7 +12533,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5a555c33e7544e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79bf69ad511f47f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12806,7 +13013,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f75ea839714bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75625661deb46f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13218,7 +13425,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf417df7c0944e34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7643106525834bac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14228,7 +14435,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24d691326bc46fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R368b56d71486465d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21710,7 +21917,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R154696f7f2e744a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd23e19e91c24383"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>